<commit_message>
Fix USDA forecast pre-fill via session state pre-seeding; add TTL to forecast config cache
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Corn Exporter Dashboard Data.xlsx
+++ b/Corn Exporter Dashboard Data.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="29" documentId="11_D631C34DEBBE4D53AC4D03116B56596AF0A43145" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8C405880-0318-44EB-82A9-8492BFC2AF50}"/>
   <bookViews>
-    <workbookView xWindow="28755" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Corn" sheetId="1" r:id="rId1"/>
@@ -9479,7 +9479,7 @@
         <v>1004.730873</v>
       </c>
       <c r="G130" s="31">
-        <f t="shared" ref="G130:G161" si="8">E130+F130</f>
+        <f t="shared" ref="G130:G140" si="8">E130+F130</f>
         <v>14425.048873</v>
       </c>
       <c r="H130" s="29">
@@ -21579,6 +21579,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="1f7db2c8-69c4-412b-9d44-16b2d9ce1096">
@@ -21587,15 +21596,6 @@
     <TaxCatchAll xmlns="2ae6f4a5-fc03-40a6-a6be-1c00f8eb7500" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -21860,20 +21860,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{18313436-0D0C-4509-B8F8-BF1D4EE350A4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D9213AC2-6ABA-48F9-BC15-50FCD621F115}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="1f7db2c8-69c4-412b-9d44-16b2d9ce1096"/>
     <ds:schemaRef ds:uri="2ae6f4a5-fc03-40a6-a6be-1c00f8eb7500"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{18313436-0D0C-4509-B8F8-BF1D4EE350A4}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Add US Census GATS + FGIS blended data feed for US export tiles
- Replace broken USDA FAS ESR API with Census Bureau International Trade API
  (api.census.gov/data/timeseries/intltrade/exports/hs) using confirmed
  Schedule B HS10 codes for corn, soybeans, soybean meal, and wheat
- Blend: GATS (official, 6-8 wk lag) primary + FGIS Socrata inspections
  forward-fill for most recent unconfirmed months
- Fix CTY_CODE=0000 issue: omit country from GET list to get world aggregates
- Handle mixed T (metric tons) and KG units across HS10 codes
- Remove Excel debug expander from sidebar

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Corn Exporter Dashboard Data.xlsx
+++ b/Corn Exporter Dashboard Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jpsicom.sharepoint.com/sites/jsacore/Shared Documents/Research Analyst/Dashboards/Corn by Major Exports/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="29" documentId="11_D631C34DEBBE4D53AC4D03116B56596AF0A43145" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8C405880-0318-44EB-82A9-8492BFC2AF50}"/>
+  <xr:revisionPtr revIDLastSave="76" documentId="11_D631C34DEBBE4D53AC4D03116B56596AF0A43145" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E32570C4-505F-4F66-8906-C39E08A84C83}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28755" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Corn" sheetId="1" r:id="rId1"/>
@@ -506,7 +506,7 @@
     <xf numFmtId="43" fontId="7" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -660,6 +660,7 @@
     <xf numFmtId="0" fontId="12" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -5175,22 +5176,22 @@
       <c r="D139" s="66">
         <v>7286</v>
       </c>
-      <c r="E139" s="67">
-        <v>155</v>
+      <c r="E139">
+        <v>477.88889</v>
       </c>
       <c r="F139" s="67">
         <v>4322</v>
       </c>
-      <c r="G139" s="66">
-        <v>2700</v>
+      <c r="G139" s="71">
+        <v>2687.4009999999998</v>
       </c>
       <c r="H139" s="68">
         <f t="shared" si="4"/>
-        <v>7177</v>
+        <v>7487.28989</v>
       </c>
       <c r="I139" s="69">
         <f t="shared" si="5"/>
-        <v>14463</v>
+        <v>14773.28989</v>
       </c>
     </row>
     <row r="140" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -9792,19 +9793,19 @@
       <c r="D140" s="19">
         <v>2988</v>
       </c>
-      <c r="E140" s="19">
-        <v>17000</v>
+      <c r="E140" s="71">
+        <v>16765.03</v>
       </c>
       <c r="F140" s="19">
         <v>0</v>
       </c>
       <c r="G140" s="60">
         <f t="shared" si="8"/>
-        <v>17000</v>
+        <v>16765.03</v>
       </c>
       <c r="H140" s="61">
         <f t="shared" si="9"/>
-        <v>19988</v>
+        <v>19753.03</v>
       </c>
       <c r="I140" s="19"/>
       <c r="J140" s="32"/>
@@ -12750,8 +12751,8 @@
       <c r="D146" s="19">
         <v>1250</v>
       </c>
-      <c r="E146" s="19">
-        <v>2274</v>
+      <c r="E146" s="71">
+        <v>2393.3220000000001</v>
       </c>
       <c r="F146" s="19">
         <v>2100</v>
@@ -12831,7 +12832,7 @@
       </c>
       <c r="F2" s="9"/>
       <c r="G2" s="9">
-        <v>1029.8583209999999</v>
+        <v>0</v>
       </c>
       <c r="H2" s="9">
         <v>240.45099999999999</v>
@@ -12859,7 +12860,7 @@
       </c>
       <c r="F3" s="9"/>
       <c r="G3" s="9">
-        <v>606.37652600000001</v>
+        <v>0</v>
       </c>
       <c r="H3" s="9">
         <v>460.113</v>
@@ -12887,7 +12888,7 @@
       </c>
       <c r="F4" s="9"/>
       <c r="G4" s="9">
-        <v>818.07181300000002</v>
+        <v>0</v>
       </c>
       <c r="H4" s="9">
         <v>416.15899999999999</v>
@@ -12918,7 +12919,7 @@
         <v>0.02</v>
       </c>
       <c r="G5" s="9">
-        <v>490.60721000000001</v>
+        <v>0.02</v>
       </c>
       <c r="H5" s="9">
         <v>512.64</v>
@@ -12949,7 +12950,7 @@
         <v>9.9760000000000009</v>
       </c>
       <c r="G6" s="9">
-        <v>703.22652000000005</v>
+        <v>9.9760000000000009</v>
       </c>
       <c r="H6" s="9">
         <v>605.89800000000002</v>
@@ -12980,7 +12981,7 @@
         <v>36.379192000000003</v>
       </c>
       <c r="G7" s="9">
-        <v>706.42052999999999</v>
+        <v>36.379192000000003</v>
       </c>
       <c r="H7" s="9">
         <v>597.92399999999998</v>
@@ -13011,7 +13012,7 @@
         <v>12.28739</v>
       </c>
       <c r="G8" s="9">
-        <v>580.05633</v>
+        <v>12.28739</v>
       </c>
       <c r="H8" s="9">
         <v>541.51099999999997</v>
@@ -13042,7 +13043,7 @@
         <v>227.09886299999999</v>
       </c>
       <c r="G9" s="9">
-        <v>723.75759000000005</v>
+        <v>227.09886299999999</v>
       </c>
       <c r="H9" s="9">
         <v>1141.126</v>
@@ -13073,7 +13074,7 @@
         <v>505.42422599999998</v>
       </c>
       <c r="G10" s="9">
-        <v>678.61572899999999</v>
+        <v>505.42422599999998</v>
       </c>
       <c r="H10" s="9">
         <v>1335.028</v>
@@ -13104,7 +13105,7 @@
         <v>613.68387099999995</v>
       </c>
       <c r="G11" s="9">
-        <v>862.39121999999998</v>
+        <v>613.68387099999995</v>
       </c>
       <c r="H11" s="9">
         <v>1359.4939999999999</v>
@@ -13135,7 +13136,7 @@
         <v>592.71981200000005</v>
       </c>
       <c r="G12" s="9">
-        <v>1111.9598410000001</v>
+        <v>592.71981200000005</v>
       </c>
       <c r="H12" s="9">
         <v>1130.8009999999999</v>
@@ -13166,7 +13167,7 @@
         <v>556.09164699999997</v>
       </c>
       <c r="G13" s="9">
-        <v>1672.6240170000001</v>
+        <v>556.09164699999997</v>
       </c>
       <c r="H13" s="9">
         <v>887.27800000000002</v>
@@ -13197,7 +13198,7 @@
         <v>333.91664200000002</v>
       </c>
       <c r="G14" s="9">
-        <v>2334.0324000000001</v>
+        <v>333.91664200000002</v>
       </c>
       <c r="H14" s="9">
         <v>785.50099999999998</v>
@@ -13227,7 +13228,7 @@
         <v>243.95169200000001</v>
       </c>
       <c r="G15" s="9">
-        <v>1762.7716379999999</v>
+        <v>243.95169200000001</v>
       </c>
       <c r="H15" s="9">
         <v>696.17100000000005</v>
@@ -13257,7 +13258,7 @@
         <v>296.18801000000002</v>
       </c>
       <c r="G16" s="9">
-        <v>1194.095333</v>
+        <v>296.18801000000002</v>
       </c>
       <c r="H16" s="9">
         <v>1057.8209999999999</v>
@@ -13287,7 +13288,7 @@
         <v>353.54237799999999</v>
       </c>
       <c r="G17" s="9">
-        <v>870.26947800000005</v>
+        <v>353.54237799999999</v>
       </c>
       <c r="H17" s="9">
         <v>1046.165</v>
@@ -13317,7 +13318,7 @@
         <v>321.53595899999999</v>
       </c>
       <c r="G18" s="9">
-        <v>742.55642399999999</v>
+        <v>321.53595899999999</v>
       </c>
       <c r="H18" s="9">
         <v>1123.606</v>
@@ -13347,7 +13348,7 @@
         <v>319.63077500000003</v>
       </c>
       <c r="G19" s="9">
-        <v>434.69002</v>
+        <v>319.63077500000003</v>
       </c>
       <c r="H19" s="9">
         <v>1095.8579999999999</v>
@@ -13377,7 +13378,7 @@
         <v>233.23755499999999</v>
       </c>
       <c r="G20" s="9">
-        <v>510.77873</v>
+        <v>233.23755499999999</v>
       </c>
       <c r="H20" s="9">
         <v>675.45100000000002</v>
@@ -13407,7 +13408,7 @@
         <v>582.77645900000005</v>
       </c>
       <c r="G21" s="9">
-        <v>489.13188500000001</v>
+        <v>582.77645900000005</v>
       </c>
       <c r="H21" s="9">
         <v>737.99400000000003</v>
@@ -13437,7 +13438,7 @@
         <v>815.80679199999997</v>
       </c>
       <c r="G22" s="9">
-        <v>370.04809</v>
+        <v>815.80679199999997</v>
       </c>
       <c r="H22" s="9">
         <v>890.78</v>
@@ -13467,7 +13468,7 @@
         <v>931.19248300000004</v>
       </c>
       <c r="G23" s="9">
-        <v>393.488</v>
+        <v>931.19248300000004</v>
       </c>
       <c r="H23" s="9">
         <v>1051.204</v>
@@ -13497,7 +13498,7 @@
         <v>859.97891000000004</v>
       </c>
       <c r="G24" s="9">
-        <v>515.18483000000003</v>
+        <v>859.97891000000004</v>
       </c>
       <c r="H24" s="9">
         <v>996.89499999999998</v>
@@ -13527,7 +13528,7 @@
         <v>717.722579</v>
       </c>
       <c r="G25" s="9">
-        <v>814.09865500000001</v>
+        <v>717.722579</v>
       </c>
       <c r="H25" s="9">
         <v>1170.4659999999999</v>
@@ -13557,7 +13558,7 @@
         <v>167.836907</v>
       </c>
       <c r="G26" s="9">
-        <v>971.73294199999998</v>
+        <v>167.836907</v>
       </c>
       <c r="H26" s="9">
         <v>1414.9690000000001</v>
@@ -13587,7 +13588,7 @@
         <v>325.37993999999998</v>
       </c>
       <c r="G27" s="9">
-        <v>647.13853099999994</v>
+        <v>325.37993999999998</v>
       </c>
       <c r="H27" s="9">
         <v>940.28099999999995</v>
@@ -13617,7 +13618,7 @@
         <v>368.34657499999997</v>
       </c>
       <c r="G28" s="9">
-        <v>842.56144099999995</v>
+        <v>368.34657499999997</v>
       </c>
       <c r="H28" s="9">
         <v>1351.848</v>
@@ -13647,7 +13648,7 @@
         <v>477.154944</v>
       </c>
       <c r="G29" s="9">
-        <v>499.146816</v>
+        <v>477.154944</v>
       </c>
       <c r="H29" s="9">
         <v>1169.1969999999999</v>
@@ -13677,7 +13678,7 @@
         <v>438.79064699999998</v>
       </c>
       <c r="G30" s="9">
-        <v>803.57628699999998</v>
+        <v>438.79064699999998</v>
       </c>
       <c r="H30" s="9">
         <v>1598.0650000000001</v>
@@ -13707,7 +13708,7 @@
         <v>509.14195699999999</v>
       </c>
       <c r="G31" s="9">
-        <v>845.54270299999996</v>
+        <v>509.14195699999999</v>
       </c>
       <c r="H31" s="9">
         <v>1171.5160000000001</v>
@@ -13737,7 +13738,7 @@
         <v>324.13772799999998</v>
       </c>
       <c r="G32" s="9">
-        <v>728.35008300000004</v>
+        <v>324.13772799999998</v>
       </c>
       <c r="H32" s="9">
         <v>803.81399999999996</v>
@@ -13767,7 +13768,7 @@
         <v>459.53978799999999</v>
       </c>
       <c r="G33" s="9">
-        <v>801.16757900000005</v>
+        <v>459.53978799999999</v>
       </c>
       <c r="H33" s="9">
         <v>1289.1969999999999</v>
@@ -13797,7 +13798,7 @@
         <v>850.87273100000004</v>
       </c>
       <c r="G34" s="9">
-        <v>508.77193999999997</v>
+        <v>850.87273100000004</v>
       </c>
       <c r="H34" s="9">
         <v>1320.4949999999999</v>
@@ -13827,7 +13828,7 @@
         <v>389.07376299999999</v>
       </c>
       <c r="G35" s="9">
-        <v>704.17954399999996</v>
+        <v>389.07376299999999</v>
       </c>
       <c r="H35" s="9">
         <v>1243.454</v>
@@ -13857,7 +13858,7 @@
         <v>168.95578800000001</v>
       </c>
       <c r="G36" s="9">
-        <v>698.58403499999997</v>
+        <v>168.95578800000001</v>
       </c>
       <c r="H36" s="9">
         <v>1183.4159999999999</v>
@@ -13887,7 +13888,7 @@
         <v>188.69044099999999</v>
       </c>
       <c r="G37" s="9">
-        <v>1647.0160550000001</v>
+        <v>188.69044099999999</v>
       </c>
       <c r="H37" s="9">
         <v>1043.7049999999999</v>
@@ -13917,7 +13918,7 @@
         <v>0</v>
       </c>
       <c r="G38" s="9">
-        <v>1441.474068</v>
+        <v>0</v>
       </c>
       <c r="H38" s="9">
         <v>1239.579</v>
@@ -13947,7 +13948,7 @@
         <v>19.152239999999999</v>
       </c>
       <c r="G39" s="9">
-        <v>1225.667631</v>
+        <v>19.152239999999999</v>
       </c>
       <c r="H39" s="9">
         <v>981.85400000000004</v>
@@ -13977,7 +13978,7 @@
         <v>52.644621000000001</v>
       </c>
       <c r="G40" s="9">
-        <v>1070.80637</v>
+        <v>52.644621000000001</v>
       </c>
       <c r="H40" s="9">
         <v>853.74199999999996</v>
@@ -14007,7 +14008,7 @@
         <v>100.565206</v>
       </c>
       <c r="G41" s="9">
-        <v>1020.003992</v>
+        <v>100.565206</v>
       </c>
       <c r="H41" s="9">
         <v>759.48699999999997</v>
@@ -14037,7 +14038,7 @@
         <v>40.361372000000003</v>
       </c>
       <c r="G42" s="9">
-        <v>688.39822500000002</v>
+        <v>40.361372000000003</v>
       </c>
       <c r="H42" s="9">
         <v>768.74300000000005</v>
@@ -14067,7 +14068,7 @@
         <v>732.46493199999998</v>
       </c>
       <c r="G43" s="9">
-        <v>684.61388999999997</v>
+        <v>732.46493199999998</v>
       </c>
       <c r="H43" s="9">
         <v>657.97699999999998</v>
@@ -14097,7 +14098,7 @@
         <v>105.911275</v>
       </c>
       <c r="G44" s="9">
-        <v>616.68786</v>
+        <v>105.911275</v>
       </c>
       <c r="H44" s="9">
         <v>712.95399999999995</v>
@@ -14127,7 +14128,7 @@
         <v>3.5264000000000002</v>
       </c>
       <c r="G45" s="9">
-        <v>384.49509</v>
+        <v>3.5264000000000002</v>
       </c>
       <c r="H45" s="9">
         <v>873.36099999999999</v>
@@ -14157,7 +14158,7 @@
         <v>1.04637</v>
       </c>
       <c r="G46" s="9">
-        <v>119.72373</v>
+        <v>1.04637</v>
       </c>
       <c r="H46" s="9">
         <v>747.529</v>
@@ -14187,7 +14188,7 @@
         <v>0.14399999999999999</v>
       </c>
       <c r="G47" s="9">
-        <v>62.425154999999997</v>
+        <v>0.14399999999999999</v>
       </c>
       <c r="H47" s="9">
         <v>706.68499999999995</v>
@@ -14217,7 +14218,7 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="G48" s="9">
-        <v>488.93956500000002</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="H48" s="9">
         <v>677.86300000000006</v>
@@ -14247,7 +14248,7 @@
         <v>0</v>
       </c>
       <c r="G49" s="9">
-        <v>1842.254545</v>
+        <v>0</v>
       </c>
       <c r="H49" s="9">
         <v>480.34899999999999</v>
@@ -14277,7 +14278,7 @@
         <v>0</v>
       </c>
       <c r="G50" s="9">
-        <v>3372.2331840000002</v>
+        <v>0</v>
       </c>
       <c r="H50" s="9">
         <v>631.80499999999995</v>
@@ -14307,7 +14308,7 @@
         <v>1.1940999999999999</v>
       </c>
       <c r="G51" s="9">
-        <v>1746.5658109999999</v>
+        <v>1.1940999999999999</v>
       </c>
       <c r="H51" s="9">
         <v>837.35599999999999</v>
@@ -14337,7 +14338,7 @@
         <v>153.06711999999999</v>
       </c>
       <c r="G52" s="9">
-        <v>10.241186000000001</v>
+        <v>153.06711999999999</v>
       </c>
       <c r="H52" s="9">
         <v>1044.6410000000001</v>
@@ -14367,7 +14368,7 @@
         <v>21.996776000000001</v>
       </c>
       <c r="G53" s="9">
-        <v>5.9724009999999996</v>
+        <v>21.996776000000001</v>
       </c>
       <c r="H53" s="9">
         <v>1620.856</v>
@@ -14397,7 +14398,7 @@
         <v>140.67432199999999</v>
       </c>
       <c r="G54" s="9">
-        <v>3.4716300000000002</v>
+        <v>140.67432199999999</v>
       </c>
       <c r="H54" s="9">
         <v>1248.5840000000001</v>
@@ -14427,7 +14428,7 @@
         <v>483.59571499999998</v>
       </c>
       <c r="G55" s="9">
-        <v>94.968905000000007</v>
+        <v>483.59571499999998</v>
       </c>
       <c r="H55" s="9">
         <v>1195.8810000000001</v>
@@ -14457,7 +14458,7 @@
         <v>645.91103199999998</v>
       </c>
       <c r="G56" s="9">
-        <v>115.26214</v>
+        <v>645.91103199999998</v>
       </c>
       <c r="H56" s="9">
         <v>1222.048</v>
@@ -14487,7 +14488,7 @@
         <v>907.86192200000005</v>
       </c>
       <c r="G57" s="9">
-        <v>462.45934799999998</v>
+        <v>907.86192200000005</v>
       </c>
       <c r="H57" s="9">
         <v>1826.5160000000001</v>
@@ -14517,7 +14518,7 @@
         <v>1542.17283</v>
       </c>
       <c r="G58" s="9">
-        <v>891.43461500000001</v>
+        <v>1542.17283</v>
       </c>
       <c r="H58" s="9">
         <v>2482.788</v>
@@ -14547,7 +14548,7 @@
         <v>1333.899733</v>
       </c>
       <c r="G59" s="9">
-        <v>621.72833000000003</v>
+        <v>1333.899733</v>
       </c>
       <c r="H59" s="9">
         <v>2843.9650000000001</v>
@@ -14577,7 +14578,7 @@
         <v>1237.604073</v>
       </c>
       <c r="G60" s="9">
-        <v>599.76840400000003</v>
+        <v>1237.604073</v>
       </c>
       <c r="H60" s="9">
         <v>1999.6320000000001</v>
@@ -14607,7 +14608,7 @@
         <v>1043.3219650000001</v>
       </c>
       <c r="G61" s="9">
-        <v>848.15759000000003</v>
+        <v>1043.3219650000001</v>
       </c>
       <c r="H61" s="9">
         <v>1699.297</v>
@@ -14637,7 +14638,7 @@
         <v>663.05717500000003</v>
       </c>
       <c r="G62" s="9">
-        <v>1167.7414739999999</v>
+        <v>663.05717500000003</v>
       </c>
       <c r="H62" s="9">
         <v>1551.2239999999999</v>
@@ -14667,7 +14668,7 @@
         <v>1045.416845</v>
       </c>
       <c r="G63" s="9">
-        <v>1107.0681099999999</v>
+        <v>1045.416845</v>
       </c>
       <c r="H63" s="9">
         <v>1816.13</v>
@@ -14697,7 +14698,7 @@
         <v>1103.66893</v>
       </c>
       <c r="G64" s="9">
-        <v>519.96947499999999</v>
+        <v>1103.66893</v>
       </c>
       <c r="H64" s="9">
         <v>2325.69</v>
@@ -14727,7 +14728,7 @@
         <v>1220.7162310000001</v>
       </c>
       <c r="G65" s="9">
-        <v>460.28032000000002</v>
+        <v>1220.7162310000001</v>
       </c>
       <c r="H65" s="9">
         <v>2052.3620000000001</v>
@@ -14757,7 +14758,7 @@
         <v>1081.793825</v>
       </c>
       <c r="G66" s="9">
-        <v>331.23043000000001</v>
+        <v>1081.793825</v>
       </c>
       <c r="H66" s="9">
         <v>1722.172</v>
@@ -14787,7 +14788,7 @@
         <v>834.92060800000002</v>
       </c>
       <c r="G67" s="9">
-        <v>180.436995</v>
+        <v>834.92060800000002</v>
       </c>
       <c r="H67" s="9">
         <v>2209.8530000000001</v>
@@ -14817,7 +14818,7 @@
         <v>592.84355000000005</v>
       </c>
       <c r="G68" s="9">
-        <v>67.640294999999995</v>
+        <v>592.84355000000005</v>
       </c>
       <c r="H68" s="9">
         <v>1622.509</v>
@@ -14847,7 +14848,7 @@
         <v>1148.982647</v>
       </c>
       <c r="G69" s="9">
-        <v>34.760415000000002</v>
+        <v>1148.982647</v>
       </c>
       <c r="H69" s="9">
         <v>1696.6959999999999</v>
@@ -14877,7 +14878,7 @@
         <v>1793.2316000000001</v>
       </c>
       <c r="G70" s="9">
-        <v>0.516629</v>
+        <v>1793.2316000000001</v>
       </c>
       <c r="H70" s="9">
         <v>2018.924</v>
@@ -14907,7 +14908,7 @@
         <v>1248.1419410000001</v>
       </c>
       <c r="G71" s="9">
-        <v>213.17987199999999</v>
+        <v>1248.1419410000001</v>
       </c>
       <c r="H71" s="9">
         <v>1835.94</v>
@@ -14937,7 +14938,7 @@
         <v>935.97428300000001</v>
       </c>
       <c r="G72" s="9">
-        <v>486.163723</v>
+        <v>935.97428300000001</v>
       </c>
       <c r="H72" s="9">
         <v>1200.7470000000001</v>
@@ -14967,7 +14968,7 @@
         <v>1036.102631</v>
       </c>
       <c r="G73" s="9">
-        <v>549.01935500000002</v>
+        <v>1036.102631</v>
       </c>
       <c r="H73" s="9">
         <v>1420.845</v>
@@ -14996,8 +14997,8 @@
       <c r="F74" s="9">
         <v>608.66269999999997</v>
       </c>
-      <c r="G74" s="9">
-        <v>571.236898</v>
+      <c r="G74" s="52">
+        <v>608.66269999999997</v>
       </c>
       <c r="H74" s="9">
         <v>1560.154</v>
@@ -15028,8 +15029,8 @@
       <c r="F75" s="9">
         <v>318.22896700000001</v>
       </c>
-      <c r="G75" s="9">
-        <v>420.48719999999997</v>
+      <c r="G75" s="52">
+        <v>318.22896700000001</v>
       </c>
       <c r="H75" s="9">
         <v>1866.299</v>
@@ -15060,8 +15061,8 @@
       <c r="F76" s="9">
         <v>544.94771600000001</v>
       </c>
-      <c r="G76" s="9">
-        <v>316.34187100000003</v>
+      <c r="G76" s="52">
+        <v>544.94771600000001</v>
       </c>
       <c r="H76" s="9">
         <v>1851.7550000000001</v>
@@ -15092,8 +15093,8 @@
       <c r="F77" s="9">
         <v>337.83063900000002</v>
       </c>
-      <c r="G77" s="9">
-        <v>438.16073</v>
+      <c r="G77" s="52">
+        <v>337.83063900000002</v>
       </c>
       <c r="H77" s="9">
         <v>1832.308</v>
@@ -15124,8 +15125,8 @@
       <c r="F78" s="9">
         <v>231.90591699999999</v>
       </c>
-      <c r="G78" s="9">
-        <v>411.29309499999999</v>
+      <c r="G78" s="52">
+        <v>231.90591699999999</v>
       </c>
       <c r="H78" s="9">
         <v>1784.8989999999999</v>
@@ -15156,8 +15157,8 @@
       <c r="F79" s="9">
         <v>204.652579</v>
       </c>
-      <c r="G79" s="9">
-        <v>444.75707499999999</v>
+      <c r="G79" s="52">
+        <v>204.652579</v>
       </c>
       <c r="H79" s="9">
         <v>1954.54</v>
@@ -15188,8 +15189,8 @@
       <c r="F80" s="9">
         <v>217.94442699999999</v>
       </c>
-      <c r="G80" s="9">
-        <v>253.34020000000001</v>
+      <c r="G80" s="52">
+        <v>217.94442699999999</v>
       </c>
       <c r="H80" s="9">
         <v>1275.9280000000001</v>
@@ -15220,8 +15221,8 @@
       <c r="F81" s="9">
         <v>422.91309699999999</v>
       </c>
-      <c r="G81" s="9">
-        <v>140.92142999999999</v>
+      <c r="G81" s="52">
+        <v>422.91309699999999</v>
       </c>
       <c r="H81" s="9">
         <v>1440.201</v>
@@ -15252,8 +15253,8 @@
       <c r="F82" s="9">
         <v>608.31982100000005</v>
       </c>
-      <c r="G82" s="9">
-        <v>147.52524</v>
+      <c r="G82" s="52">
+        <v>608.31982100000005</v>
       </c>
       <c r="H82" s="9">
         <v>2955.652</v>
@@ -15284,8 +15285,8 @@
       <c r="F83" s="9">
         <v>753.95514600000001</v>
       </c>
-      <c r="G83" s="9">
-        <v>75.022194999999996</v>
+      <c r="G83" s="52">
+        <v>753.95514600000001</v>
       </c>
       <c r="H83" s="9">
         <v>2335.9780000000001</v>
@@ -15316,8 +15317,8 @@
       <c r="F84" s="9">
         <v>195.079622</v>
       </c>
-      <c r="G84" s="9">
-        <v>53.844700000000003</v>
+      <c r="G84" s="52">
+        <v>195.079622</v>
       </c>
       <c r="H84" s="9">
         <v>2321.3090000000002</v>
@@ -15348,8 +15349,8 @@
       <c r="F85" s="9">
         <v>361.723929</v>
       </c>
-      <c r="G85" s="9">
-        <v>766.06604500000003</v>
+      <c r="G85" s="52">
+        <v>361.723929</v>
       </c>
       <c r="H85" s="9">
         <v>1521.1880000000001</v>
@@ -15380,8 +15381,8 @@
       <c r="F86" s="9">
         <v>37.055390000000003</v>
       </c>
-      <c r="G86" s="9">
-        <v>1124.6281690000001</v>
+      <c r="G86" s="52">
+        <v>37.055390000000003</v>
       </c>
       <c r="H86" s="9">
         <v>1347.9490000000001</v>
@@ -15412,8 +15413,8 @@
       <c r="F87" s="9">
         <v>193.94697099999999</v>
       </c>
-      <c r="G87" s="9">
-        <v>1156.3569809999999</v>
+      <c r="G87" s="52">
+        <v>193.94697099999999</v>
       </c>
       <c r="H87" s="9">
         <v>1620.752</v>
@@ -15444,8 +15445,8 @@
       <c r="F88" s="9">
         <v>322.60136799999998</v>
       </c>
-      <c r="G88" s="9">
-        <v>984.884908</v>
+      <c r="G88" s="52">
+        <v>322.60136799999998</v>
       </c>
       <c r="H88" s="9">
         <v>2439.6970000000001</v>
@@ -15476,8 +15477,8 @@
       <c r="F89" s="9">
         <v>152.73443800000001</v>
       </c>
-      <c r="G89" s="9">
-        <v>636.04062999999996</v>
+      <c r="G89" s="52">
+        <v>152.73443800000001</v>
       </c>
       <c r="H89" s="9">
         <v>1344.355</v>
@@ -15508,8 +15509,8 @@
       <c r="F90" s="9">
         <v>72.595982000000006</v>
       </c>
-      <c r="G90" s="9">
-        <v>479.992345</v>
+      <c r="G90" s="52">
+        <v>72.595982000000006</v>
       </c>
       <c r="H90" s="9">
         <v>1565.721</v>
@@ -15540,8 +15541,8 @@
       <c r="F91" s="9">
         <v>806.27274299999999</v>
       </c>
-      <c r="G91" s="9">
-        <v>588.28198699999996</v>
+      <c r="G91" s="52">
+        <v>806.27274299999999</v>
       </c>
       <c r="H91" s="9">
         <v>1113.846</v>
@@ -15572,8 +15573,8 @@
       <c r="F92" s="9">
         <v>136.99258599999999</v>
       </c>
-      <c r="G92" s="9">
-        <v>377.98827499999999</v>
+      <c r="G92" s="52">
+        <v>136.99258599999999</v>
       </c>
       <c r="H92" s="9">
         <v>1022.072</v>
@@ -15604,8 +15605,8 @@
       <c r="F93" s="9">
         <v>567.21168</v>
       </c>
-      <c r="G93" s="9">
-        <v>629.14156300000002</v>
+      <c r="G93" s="52">
+        <v>567.21168</v>
       </c>
       <c r="H93" s="9">
         <v>1198.585</v>
@@ -15636,8 +15637,8 @@
       <c r="F94" s="9">
         <v>830.18803300000002</v>
       </c>
-      <c r="G94" s="9">
-        <v>488.35017800000003</v>
+      <c r="G94" s="52">
+        <v>830.18803300000002</v>
       </c>
       <c r="H94" s="9">
         <v>1837.8119999999999</v>
@@ -15668,8 +15669,8 @@
       <c r="F95" s="9">
         <v>140.14698999999999</v>
       </c>
-      <c r="G95" s="9">
-        <v>451.00295999999997</v>
+      <c r="G95" s="52">
+        <v>140.14698999999999</v>
       </c>
       <c r="H95" s="9">
         <v>1485.748</v>
@@ -15700,8 +15701,8 @@
       <c r="F96" s="9">
         <v>466.28957500000001</v>
       </c>
-      <c r="G96" s="9">
-        <v>449.35233499999998</v>
+      <c r="G96" s="52">
+        <v>466.28957500000001</v>
       </c>
       <c r="H96" s="9">
         <v>1804.546</v>
@@ -15732,8 +15733,8 @@
       <c r="F97" s="9">
         <v>339.44728099999998</v>
       </c>
-      <c r="G97" s="9">
-        <v>824.00250000000005</v>
+      <c r="G97" s="52">
+        <v>339.44728099999998</v>
       </c>
       <c r="H97" s="9">
         <v>1226.2629999999999</v>
@@ -15764,8 +15765,8 @@
       <c r="F98" s="9">
         <v>362.59286900000001</v>
       </c>
-      <c r="G98" s="9">
-        <v>1363.221452</v>
+      <c r="G98" s="52">
+        <v>362.59286900000001</v>
       </c>
       <c r="H98" s="9">
         <v>1099.0450000000001</v>
@@ -15796,8 +15797,8 @@
       <c r="F99" s="9">
         <v>378.682095</v>
       </c>
-      <c r="G99" s="9">
-        <v>1447.3381710000001</v>
+      <c r="G99" s="52">
+        <v>378.682095</v>
       </c>
       <c r="H99" s="9">
         <v>949.63800000000003</v>
@@ -15828,8 +15829,8 @@
       <c r="F100" s="9">
         <v>564.73312599999997</v>
       </c>
-      <c r="G100" s="9">
-        <v>1276.964035</v>
+      <c r="G100" s="52">
+        <v>564.73312599999997</v>
       </c>
       <c r="H100" s="9">
         <v>1504.4580000000001</v>
@@ -15860,8 +15861,8 @@
       <c r="F101" s="9">
         <v>489.80265200000002</v>
       </c>
-      <c r="G101" s="9">
-        <v>1220.779415</v>
+      <c r="G101" s="52">
+        <v>489.80265200000002</v>
       </c>
       <c r="H101" s="9">
         <v>1087.1469999999999</v>
@@ -15892,8 +15893,8 @@
       <c r="F102" s="9">
         <v>599.68059800000003</v>
       </c>
-      <c r="G102" s="9">
-        <v>1062.6213499999999</v>
+      <c r="G102" s="52">
+        <v>599.68059800000003</v>
       </c>
       <c r="H102" s="9">
         <v>824.9</v>
@@ -15924,8 +15925,8 @@
       <c r="F103" s="9">
         <v>314.33884999999998</v>
       </c>
-      <c r="G103" s="9">
-        <v>986.76868999999999</v>
+      <c r="G103" s="52">
+        <v>314.33884999999998</v>
       </c>
       <c r="H103" s="9">
         <v>642.71500000000003</v>
@@ -15956,8 +15957,8 @@
       <c r="F104" s="9">
         <v>326.805361</v>
       </c>
-      <c r="G104" s="9">
-        <v>1327.41149</v>
+      <c r="G104" s="52">
+        <v>326.805361</v>
       </c>
       <c r="H104" s="9">
         <v>554.95799999999997</v>
@@ -15988,8 +15989,8 @@
       <c r="F105" s="9">
         <v>864.42854399999999</v>
       </c>
-      <c r="G105" s="9">
-        <v>779.17014500000005</v>
+      <c r="G105" s="52">
+        <v>864.42854399999999</v>
       </c>
       <c r="H105" s="9">
         <v>1347.616</v>
@@ -16020,8 +16021,8 @@
       <c r="F106" s="9">
         <v>1243.85628</v>
       </c>
-      <c r="G106" s="9">
-        <v>573.71238000000005</v>
+      <c r="G106" s="52">
+        <v>1243.85628</v>
       </c>
       <c r="H106" s="9">
         <v>1690.3409999999999</v>
@@ -16052,8 +16053,8 @@
       <c r="F107" s="9">
         <v>1502.33286</v>
       </c>
-      <c r="G107" s="9">
-        <v>453.11223100000001</v>
+      <c r="G107" s="52">
+        <v>1502.33286</v>
       </c>
       <c r="H107" s="9">
         <v>2520.8589999999999</v>
@@ -16084,8 +16085,8 @@
       <c r="F108" s="9">
         <v>1414.2530549999999</v>
       </c>
-      <c r="G108" s="9">
-        <v>301.58201500000001</v>
+      <c r="G108" s="52">
+        <v>1414.2530549999999</v>
       </c>
       <c r="H108" s="9">
         <v>2397.25</v>
@@ -16116,8 +16117,8 @@
       <c r="F109" s="9">
         <v>529.98731399999997</v>
       </c>
-      <c r="G109" s="9">
-        <v>722.92202999999995</v>
+      <c r="G109" s="52">
+        <v>529.98731399999997</v>
       </c>
       <c r="H109" s="9">
         <v>2295.6289999999999</v>
@@ -16148,8 +16149,8 @@
       <c r="F110" s="9">
         <v>122.287524</v>
       </c>
-      <c r="G110" s="9">
-        <v>722.81898000000001</v>
+      <c r="G110" s="52">
+        <v>122.287524</v>
       </c>
       <c r="H110" s="9">
         <v>1974.623</v>
@@ -16180,8 +16181,8 @@
       <c r="F111" s="9">
         <v>188.54431400000001</v>
       </c>
-      <c r="G111" s="9">
-        <v>610.40747999999996</v>
+      <c r="G111" s="52">
+        <v>188.54431400000001</v>
       </c>
       <c r="H111" s="9">
         <v>2393.81</v>
@@ -16212,8 +16213,8 @@
       <c r="F112" s="9">
         <v>64.846615999999997</v>
       </c>
-      <c r="G112" s="9">
-        <v>410.83049099999999</v>
+      <c r="G112" s="52">
+        <v>64.846615999999997</v>
       </c>
       <c r="H112" s="9">
         <v>2562.201</v>
@@ -16244,8 +16245,8 @@
       <c r="F113" s="9">
         <v>279.90608900000001</v>
       </c>
-      <c r="G113" s="9">
-        <v>306.34327500000001</v>
+      <c r="G113" s="52">
+        <v>279.90608900000001</v>
       </c>
       <c r="H113" s="9">
         <v>2164.0140000000001</v>
@@ -16276,8 +16277,8 @@
       <c r="F114" s="9">
         <v>163.93786700000001</v>
       </c>
-      <c r="G114" s="9">
-        <v>247.24195</v>
+      <c r="G114" s="52">
+        <v>163.93786700000001</v>
       </c>
       <c r="H114" s="9">
         <v>1585.0940000000001</v>
@@ -16308,8 +16309,8 @@
       <c r="F115" s="9">
         <v>129.04637299999999</v>
       </c>
-      <c r="G115" s="9">
-        <v>83.277850000000001</v>
+      <c r="G115" s="52">
+        <v>129.04637299999999</v>
       </c>
       <c r="H115" s="9">
         <v>1235.8510000000001</v>
@@ -16340,8 +16341,8 @@
       <c r="F116" s="9">
         <v>260.26202899999998</v>
       </c>
-      <c r="G116" s="9">
-        <v>0</v>
+      <c r="G116" s="52">
+        <v>260.26202899999998</v>
       </c>
       <c r="H116" s="9">
         <v>1489.4749999999999</v>
@@ -16372,8 +16373,8 @@
       <c r="F117" s="9">
         <v>1297.3640740000001</v>
       </c>
-      <c r="G117" s="9">
-        <v>0.69982999999999995</v>
+      <c r="G117" s="52">
+        <v>1297.3640740000001</v>
       </c>
       <c r="H117" s="9">
         <v>2864.5320000000002</v>
@@ -16404,8 +16405,8 @@
       <c r="F118" s="9">
         <v>1930.563703</v>
       </c>
-      <c r="G118" s="9">
-        <v>0.19900000000000001</v>
+      <c r="G118" s="52">
+        <v>1930.563703</v>
       </c>
       <c r="H118" s="9">
         <v>2869.28</v>
@@ -16436,8 +16437,8 @@
       <c r="F119" s="9">
         <v>1713.5302360000001</v>
       </c>
-      <c r="G119" s="9">
-        <v>0</v>
+      <c r="G119" s="52">
+        <v>1713.5302360000001</v>
       </c>
       <c r="H119" s="9">
         <v>2806.2979999999998</v>
@@ -16468,8 +16469,8 @@
       <c r="F120" s="9">
         <v>793.02634</v>
       </c>
-      <c r="G120" s="9">
-        <v>0</v>
+      <c r="G120" s="52">
+        <v>793.02634</v>
       </c>
       <c r="H120" s="9">
         <v>2442.2629999999999</v>
@@ -16500,8 +16501,8 @@
       <c r="F121" s="9">
         <v>792.26033199999995</v>
       </c>
-      <c r="G121" s="9">
-        <v>27.245059999999999</v>
+      <c r="G121" s="52">
+        <v>792.26033199999995</v>
       </c>
       <c r="H121" s="9">
         <v>3054.2719999999999</v>
@@ -16532,7 +16533,7 @@
       <c r="F122" s="9">
         <v>156.56712999999999</v>
       </c>
-      <c r="G122" s="9">
+      <c r="G122" s="52">
         <v>188.09502699999999</v>
       </c>
       <c r="H122" s="9">
@@ -16564,7 +16565,7 @@
       <c r="F123" s="9">
         <v>251.49464499999999</v>
       </c>
-      <c r="G123" s="9">
+      <c r="G123" s="52">
         <v>448.59676300000001</v>
       </c>
       <c r="H123" s="9">
@@ -16596,7 +16597,7 @@
       <c r="F124" s="9">
         <v>291.84381500000001</v>
       </c>
-      <c r="G124" s="9">
+      <c r="G124" s="52">
         <v>314.180792</v>
       </c>
       <c r="H124" s="9">
@@ -16628,7 +16629,7 @@
       <c r="F125" s="9">
         <v>227.86555999999999</v>
       </c>
-      <c r="G125" s="9">
+      <c r="G125" s="52">
         <v>592.52487199999996</v>
       </c>
       <c r="H125" s="9">
@@ -16660,7 +16661,7 @@
       <c r="F126" s="9">
         <v>107.92046000000001</v>
       </c>
-      <c r="G126" s="9">
+      <c r="G126" s="52">
         <v>679.20216200000004</v>
       </c>
       <c r="H126" s="9">
@@ -16692,7 +16693,7 @@
       <c r="F127" s="9">
         <v>147.57038</v>
       </c>
-      <c r="G127" s="9">
+      <c r="G127" s="52">
         <v>374.13977</v>
       </c>
       <c r="H127" s="9">
@@ -16724,7 +16725,7 @@
       <c r="F128" s="9">
         <v>147.40610000000001</v>
       </c>
-      <c r="G128" s="9">
+      <c r="G128" s="52">
         <v>622.84785099999999</v>
       </c>
       <c r="H128" s="9">
@@ -16756,7 +16757,7 @@
       <c r="F129" s="9">
         <v>24.01239</v>
       </c>
-      <c r="G129" s="9">
+      <c r="G129" s="52">
         <v>1703.599978</v>
       </c>
       <c r="H129" s="9">
@@ -16788,7 +16789,7 @@
       <c r="F130" s="9">
         <v>122.98027500000001</v>
       </c>
-      <c r="G130" s="9">
+      <c r="G130" s="52">
         <v>2181.3972469999999</v>
       </c>
       <c r="H130" s="9">
@@ -16820,7 +16821,7 @@
       <c r="F131" s="9">
         <v>38.569800000000001</v>
       </c>
-      <c r="G131" s="9">
+      <c r="G131" s="52">
         <v>1655.3360379999999</v>
       </c>
       <c r="H131" s="9">
@@ -16852,7 +16853,7 @@
       <c r="F132" s="9">
         <v>38.483049999999999</v>
       </c>
-      <c r="G132" s="9">
+      <c r="G132" s="52">
         <v>1017.396341</v>
       </c>
       <c r="H132" s="9">
@@ -16884,7 +16885,7 @@
       <c r="F133" s="9">
         <v>295.97111999999998</v>
       </c>
-      <c r="G133" s="9">
+      <c r="G133" s="52">
         <v>765.87637600000005</v>
       </c>
       <c r="H133" s="9">
@@ -16916,7 +16917,7 @@
       <c r="F134" s="9">
         <v>502.78506499999997</v>
       </c>
-      <c r="G134" s="9">
+      <c r="G134" s="52">
         <v>551.41869399999996</v>
       </c>
       <c r="H134" s="9">
@@ -16948,7 +16949,7 @@
       <c r="F135" s="9">
         <v>569.38151000000005</v>
       </c>
-      <c r="G135" s="9">
+      <c r="G135" s="52">
         <v>650.21983999999998</v>
       </c>
       <c r="H135" s="9">
@@ -16980,7 +16981,7 @@
       <c r="F136" s="9">
         <v>463.98432500000001</v>
       </c>
-      <c r="G136" s="9">
+      <c r="G136" s="52">
         <v>494.46200599999997</v>
       </c>
       <c r="H136" s="9">
@@ -17012,7 +17013,7 @@
       <c r="F137" s="9">
         <v>484.84030999999999</v>
       </c>
-      <c r="G137" s="9">
+      <c r="G137" s="52">
         <v>483.85564099999999</v>
       </c>
       <c r="H137" s="9">
@@ -17044,7 +17045,7 @@
       <c r="F138" s="9">
         <v>326.17374000000001</v>
       </c>
-      <c r="G138" s="9">
+      <c r="G138" s="52">
         <v>396.48701399999999</v>
       </c>
       <c r="H138" s="9">
@@ -17076,7 +17077,7 @@
       <c r="F139" s="9">
         <v>426.56977999999998</v>
       </c>
-      <c r="G139" s="9">
+      <c r="G139" s="52">
         <v>359.79334699999998</v>
       </c>
       <c r="H139" s="9">
@@ -17108,7 +17109,7 @@
       <c r="F140" s="9">
         <v>279.50517500000001</v>
       </c>
-      <c r="G140" s="9">
+      <c r="G140" s="52">
         <v>769.825378</v>
       </c>
       <c r="H140" s="9">
@@ -17140,7 +17141,7 @@
       <c r="F141" s="9">
         <v>375.76101599999998</v>
       </c>
-      <c r="G141" s="9">
+      <c r="G141" s="52">
         <v>1892.397393</v>
       </c>
       <c r="H141" s="9">
@@ -17172,7 +17173,7 @@
       <c r="F142" s="9">
         <v>369.41748999999999</v>
       </c>
-      <c r="G142" s="9">
+      <c r="G142" s="52">
         <v>2813.586585</v>
       </c>
       <c r="H142" s="9">
@@ -17204,7 +17205,7 @@
       <c r="F143" s="9">
         <v>293.30811999999997</v>
       </c>
-      <c r="G143" s="9">
+      <c r="G143" s="52">
         <v>2065.9993530000002</v>
       </c>
       <c r="H143" s="9">
@@ -17236,7 +17237,7 @@
       <c r="F144" s="9">
         <v>171.78908000000001</v>
       </c>
-      <c r="G144" s="9">
+      <c r="G144" s="52">
         <v>1377.836399</v>
       </c>
       <c r="H144" s="9">
@@ -17268,7 +17269,7 @@
       <c r="F145" s="9">
         <v>53.496220000000001</v>
       </c>
-      <c r="G145" s="9">
+      <c r="G145" s="52">
         <v>1594.082723</v>
       </c>
       <c r="H145" s="9">
@@ -17300,7 +17301,7 @@
       <c r="F146" s="9">
         <v>940.56795999999997</v>
       </c>
-      <c r="G146" s="9">
+      <c r="G146" s="52">
         <v>465.88551799999999</v>
       </c>
       <c r="H146" s="9">
@@ -17332,7 +17333,7 @@
       <c r="F147" s="9">
         <v>1162.922984</v>
       </c>
-      <c r="G147" s="9">
+      <c r="G147" s="52">
         <v>854.50036599999999</v>
       </c>
       <c r="H147" s="9">
@@ -17364,7 +17365,7 @@
       <c r="F148" s="9">
         <v>1454.0275340000001</v>
       </c>
-      <c r="G148" s="9">
+      <c r="G148" s="52">
         <v>1071.920192</v>
       </c>
       <c r="H148" s="9">
@@ -17396,7 +17397,7 @@
       <c r="F149" s="9">
         <v>1283.0401300000001</v>
       </c>
-      <c r="G149" s="9">
+      <c r="G149" s="52">
         <v>1317.2800139999999</v>
       </c>
       <c r="H149" s="9">
@@ -17428,7 +17429,7 @@
       <c r="F150" s="9">
         <v>907.09361999999999</v>
       </c>
-      <c r="G150" s="9">
+      <c r="G150" s="52">
         <v>1406.386448</v>
       </c>
       <c r="H150" s="9">
@@ -17460,7 +17461,7 @@
       <c r="F151" s="9">
         <v>669.13553000000002</v>
       </c>
-      <c r="G151" s="9">
+      <c r="G151" s="52">
         <v>1296.923976</v>
       </c>
       <c r="H151" s="9">
@@ -17492,7 +17493,7 @@
       <c r="F152" s="9">
         <v>529.32949499999995</v>
       </c>
-      <c r="G152" s="9">
+      <c r="G152" s="52">
         <v>726.59695399999998</v>
       </c>
       <c r="H152" s="9">
@@ -17524,7 +17525,7 @@
       <c r="F153" s="9">
         <v>459.66716000000002</v>
       </c>
-      <c r="G153" s="9">
+      <c r="G153" s="52">
         <v>3045.9776510000002</v>
       </c>
       <c r="H153" s="9">
@@ -17556,7 +17557,7 @@
       <c r="F154" s="9">
         <v>263.11822000000001</v>
       </c>
-      <c r="G154" s="9">
+      <c r="G154" s="52">
         <v>2863.5670879999998</v>
       </c>
       <c r="H154" s="9">
@@ -17588,7 +17589,7 @@
       <c r="F155" s="9">
         <v>416.95828</v>
       </c>
-      <c r="G155" s="9">
+      <c r="G155" s="52">
         <v>2057.904884</v>
       </c>
       <c r="H155" s="9">
@@ -17620,7 +17621,7 @@
       <c r="F156" s="9">
         <v>573.04407200000003</v>
       </c>
-      <c r="G156" s="9">
+      <c r="G156" s="52">
         <v>1402.0785069999999</v>
       </c>
       <c r="H156" s="9">
@@ -17652,7 +17653,7 @@
       <c r="F157" s="9">
         <v>1606.994344</v>
       </c>
-      <c r="G157" s="9">
+      <c r="G157" s="52">
         <v>1409.3035259999999</v>
       </c>
       <c r="H157" s="9">
@@ -17684,7 +17685,7 @@
       <c r="F158" s="9">
         <v>2349.4069060000002</v>
       </c>
-      <c r="G158" s="9">
+      <c r="G158" s="52">
         <v>1212.5626299999999</v>
       </c>
       <c r="H158" s="9">
@@ -17716,7 +17717,7 @@
       <c r="F159" s="9">
         <v>1991.180775</v>
       </c>
-      <c r="G159" s="9">
+      <c r="G159" s="52">
         <v>839.97423900000001</v>
       </c>
       <c r="H159" s="9">
@@ -17748,7 +17749,7 @@
       <c r="F160" s="9">
         <v>1248.2495799999999</v>
       </c>
-      <c r="G160" s="9">
+      <c r="G160" s="52">
         <v>1052.2953689999999</v>
       </c>
       <c r="H160" s="9">
@@ -17780,7 +17781,7 @@
       <c r="F161" s="9">
         <v>761.44653500000004</v>
       </c>
-      <c r="G161" s="9">
+      <c r="G161" s="52">
         <v>1198.352341</v>
       </c>
       <c r="H161" s="9">
@@ -17812,7 +17813,7 @@
       <c r="F162" s="9">
         <v>501.01107500000001</v>
       </c>
-      <c r="G162" s="9">
+      <c r="G162" s="52">
         <v>984.99572799999999</v>
       </c>
       <c r="H162" s="9">
@@ -17844,7 +17845,7 @@
       <c r="F163" s="9">
         <v>599.84281499999997</v>
       </c>
-      <c r="G163" s="9">
+      <c r="G163" s="52">
         <v>734.36431300000004</v>
       </c>
       <c r="H163" s="9">
@@ -17876,7 +17877,7 @@
       <c r="F164" s="9">
         <v>689.70649500000002</v>
       </c>
-      <c r="G164" s="9">
+      <c r="G164" s="52">
         <v>810.06392800000003</v>
       </c>
       <c r="H164" s="9">
@@ -17908,7 +17909,7 @@
       <c r="F165" s="9">
         <v>749.53636500000005</v>
       </c>
-      <c r="G165" s="9">
+      <c r="G165" s="52">
         <v>2478.2240689999999</v>
       </c>
       <c r="H165" s="9">
@@ -17940,7 +17941,7 @@
       <c r="F166" s="9">
         <v>620.82923500000004</v>
       </c>
-      <c r="G166" s="9">
+      <c r="G166" s="52">
         <v>2642.2346149999998</v>
       </c>
       <c r="H166" s="9">
@@ -17972,7 +17973,7 @@
       <c r="F167" s="9">
         <v>767.86617000000001</v>
       </c>
-      <c r="G167" s="9">
+      <c r="G167" s="52">
         <v>2261.7771670000002</v>
       </c>
       <c r="H167" s="9">
@@ -18004,7 +18005,7 @@
       <c r="F168" s="9">
         <v>929.47409000000005</v>
       </c>
-      <c r="G168" s="9">
+      <c r="G168" s="52">
         <v>1832.024713</v>
       </c>
       <c r="H168" s="9">
@@ -18036,7 +18037,7 @@
       <c r="F169" s="9">
         <v>1890.398209</v>
       </c>
-      <c r="G169" s="9">
+      <c r="G169" s="52">
         <v>1264.3922809999999</v>
       </c>
       <c r="H169" s="9">
@@ -18068,7 +18069,7 @@
       <c r="F170" s="9">
         <v>2391.316354</v>
       </c>
-      <c r="G170" s="9">
+      <c r="G170" s="52">
         <v>872.51106900000002</v>
       </c>
       <c r="H170" s="9">
@@ -18100,7 +18101,7 @@
       <c r="F171" s="9">
         <v>1746.275975</v>
       </c>
-      <c r="G171" s="9">
+      <c r="G171" s="52">
         <v>1040.234508</v>
       </c>
       <c r="H171" s="9">
@@ -18132,7 +18133,7 @@
       <c r="F172" s="9">
         <v>1631.86664</v>
       </c>
-      <c r="G172" s="9">
+      <c r="G172" s="52">
         <v>1011.641572</v>
       </c>
       <c r="H172" s="9">
@@ -18164,7 +18165,7 @@
       <c r="F173" s="9">
         <v>622.88483599999995</v>
       </c>
-      <c r="G173" s="9">
+      <c r="G173" s="52">
         <v>1123.1866210000001</v>
       </c>
       <c r="H173" s="9">
@@ -18196,7 +18197,7 @@
       <c r="F174" s="9">
         <v>607.96240999999998</v>
       </c>
-      <c r="G174" s="9">
+      <c r="G174" s="52">
         <v>1009.511436</v>
       </c>
       <c r="H174" s="9">
@@ -18228,7 +18229,7 @@
       <c r="F175" s="9">
         <v>392.21839999999997</v>
       </c>
-      <c r="G175" s="9">
+      <c r="G175" s="52">
         <v>806.62124600000004</v>
       </c>
       <c r="H175" s="9">
@@ -18260,7 +18261,7 @@
       <c r="F176" s="9">
         <v>485.88135</v>
       </c>
-      <c r="G176" s="9">
+      <c r="G176" s="52">
         <v>940.18248400000004</v>
       </c>
       <c r="H176" s="9">
@@ -18292,7 +18293,7 @@
       <c r="F177" s="9">
         <v>534.50174000000004</v>
       </c>
-      <c r="G177" s="9">
+      <c r="G177" s="52">
         <v>2171.342435</v>
       </c>
       <c r="H177" s="9">
@@ -18324,7 +18325,7 @@
       <c r="F178" s="9">
         <v>471.90320000000003</v>
       </c>
-      <c r="G178" s="9">
+      <c r="G178" s="52">
         <v>2258.5481639999998</v>
       </c>
       <c r="H178" s="9">
@@ -18356,7 +18357,7 @@
       <c r="F179" s="9">
         <v>372.04706499999998</v>
       </c>
-      <c r="G179" s="9">
+      <c r="G179" s="52">
         <v>2186.6433550000002</v>
       </c>
       <c r="H179" s="9">
@@ -18388,7 +18389,7 @@
       <c r="F180" s="9">
         <v>707.21092399999998</v>
       </c>
-      <c r="G180" s="9">
+      <c r="G180" s="52">
         <v>1852.6503319999999</v>
       </c>
       <c r="H180" s="9">
@@ -18420,7 +18421,7 @@
       <c r="F181" s="9">
         <v>2104.786118</v>
       </c>
-      <c r="G181" s="9">
+      <c r="G181" s="52">
         <v>1098.5630630000001</v>
       </c>
       <c r="H181" s="9">
@@ -18452,7 +18453,7 @@
       <c r="F182" s="9">
         <v>2700.4772889999999</v>
       </c>
-      <c r="G182" s="9">
+      <c r="G182" s="52">
         <v>1011.649279</v>
       </c>
       <c r="H182" s="9">
@@ -18484,7 +18485,7 @@
       <c r="F183" s="9">
         <v>1520.332015</v>
       </c>
-      <c r="G183" s="9">
+      <c r="G183" s="52">
         <v>971.8338</v>
       </c>
       <c r="H183" s="9">
@@ -18516,7 +18517,7 @@
       <c r="F184" s="9">
         <v>949.05609200000004</v>
       </c>
-      <c r="G184" s="9">
+      <c r="G184" s="52">
         <v>890.99006799999995</v>
       </c>
       <c r="H184" s="9">
@@ -18548,7 +18549,7 @@
       <c r="F185" s="9">
         <v>861.302548</v>
       </c>
-      <c r="G185" s="9">
+      <c r="G185" s="52">
         <v>940.90168500000004</v>
       </c>
       <c r="H185" s="9">
@@ -18580,7 +18581,7 @@
       <c r="F186" s="9">
         <v>646.54062499999998</v>
       </c>
-      <c r="G186" s="9">
+      <c r="G186" s="52">
         <v>827.04068800000005</v>
       </c>
       <c r="H186" s="9">
@@ -18612,7 +18613,7 @@
       <c r="F187" s="9">
         <v>480.97782000000001</v>
       </c>
-      <c r="G187" s="9">
+      <c r="G187" s="52">
         <v>423.87985600000002</v>
       </c>
       <c r="H187" s="9">
@@ -18644,7 +18645,7 @@
       <c r="F188" s="9">
         <v>435.74309499999998</v>
       </c>
-      <c r="G188" s="9">
+      <c r="G188" s="52">
         <v>1262.4357500000001</v>
       </c>
       <c r="H188" s="9">
@@ -18676,7 +18677,7 @@
       <c r="F189" s="9">
         <v>392.53982500000001</v>
       </c>
-      <c r="G189" s="9">
+      <c r="G189" s="52">
         <v>3548.1182450000001</v>
       </c>
       <c r="H189" s="9">
@@ -18708,7 +18709,7 @@
       <c r="F190" s="9">
         <v>301.94991499999998</v>
       </c>
-      <c r="G190" s="9">
+      <c r="G190" s="52">
         <v>3814.6222389999998</v>
       </c>
       <c r="H190" s="9">
@@ -18740,7 +18741,7 @@
       <c r="F191" s="9">
         <v>231.57137</v>
       </c>
-      <c r="G191" s="9">
+      <c r="G191" s="52">
         <v>2905.3951849999999</v>
       </c>
       <c r="H191" s="9">
@@ -18772,7 +18773,7 @@
       <c r="F192" s="9">
         <v>667.415978</v>
       </c>
-      <c r="G192" s="9">
+      <c r="G192" s="52">
         <v>1938.133493</v>
       </c>
       <c r="H192" s="9">
@@ -18804,7 +18805,7 @@
       <c r="F193" s="9">
         <v>2103.5420800000002</v>
       </c>
-      <c r="G193" s="9">
+      <c r="G193" s="52">
         <v>1486.767155</v>
       </c>
       <c r="H193" s="9">
@@ -19221,7 +19222,7 @@
         <v>507.69638600000002</v>
       </c>
       <c r="G206" s="9">
-        <v>401.08499799999998</v>
+        <v>507.69638600000002</v>
       </c>
       <c r="H206" s="9">
         <v>2207.1999999999998</v>
@@ -19253,7 +19254,7 @@
         <v>708.99805300000003</v>
       </c>
       <c r="G207" s="9">
-        <v>121.330839</v>
+        <v>708.99805300000003</v>
       </c>
       <c r="H207" s="9">
         <v>2603.2170000000001</v>
@@ -19285,7 +19286,7 @@
         <v>696.95005600000002</v>
       </c>
       <c r="G208" s="9">
-        <v>45.341512999999999</v>
+        <v>696.95005600000002</v>
       </c>
       <c r="H208" s="9">
         <v>2612.9870000000001</v>
@@ -19317,7 +19318,7 @@
         <v>713.19848200000001</v>
       </c>
       <c r="G209" s="9">
-        <v>0</v>
+        <v>713.19848200000001</v>
       </c>
       <c r="H209" s="9">
         <v>2276.9050000000002</v>
@@ -19349,7 +19350,7 @@
         <v>857.66653099999996</v>
       </c>
       <c r="G210" s="9">
-        <v>1.0000000000000001E-5</v>
+        <v>857.66653099999996</v>
       </c>
       <c r="H210" s="9">
         <v>1955.9190000000001</v>
@@ -19381,7 +19382,7 @@
         <v>662.23156700000004</v>
       </c>
       <c r="G211" s="9">
-        <v>0</v>
+        <v>662.23156700000004</v>
       </c>
       <c r="H211" s="9">
         <v>987.35199999999998</v>
@@ -19413,7 +19414,7 @@
         <v>960.59852999999998</v>
       </c>
       <c r="G212" s="9">
-        <v>1.9999999999999999E-6</v>
+        <v>960.59852999999998</v>
       </c>
       <c r="H212" s="9">
         <v>1640.855</v>
@@ -19445,7 +19446,7 @@
         <v>3612.050565</v>
       </c>
       <c r="G213" s="9">
-        <v>21.014759999999999</v>
+        <v>3612.050565</v>
       </c>
       <c r="H213" s="9">
         <v>3645.2370000000001</v>
@@ -19477,7 +19478,7 @@
         <v>4362.9818580000001</v>
       </c>
       <c r="G214" s="9">
-        <v>1.5E-5</v>
+        <v>4362.9818580000001</v>
       </c>
       <c r="H214" s="9">
         <v>4169.6019999999999</v>
@@ -19509,7 +19510,7 @@
         <v>3414.9189240000001</v>
       </c>
       <c r="G215" s="9">
-        <v>0</v>
+        <v>3414.9189240000001</v>
       </c>
       <c r="H215" s="9">
         <v>2445.9</v>
@@ -19541,7 +19542,7 @@
         <v>2375.0333860000001</v>
       </c>
       <c r="G216" s="9">
-        <v>2.8E-5</v>
+        <v>2375.0333860000001</v>
       </c>
       <c r="H216" s="9">
         <v>2202.5859999999998</v>
@@ -19573,7 +19574,7 @@
         <v>1173.06522</v>
       </c>
       <c r="G217" s="9">
-        <v>540.51514999999995</v>
+        <v>1173.06522</v>
       </c>
       <c r="H217" s="9">
         <v>2227.989</v>
@@ -19605,7 +19606,7 @@
         <v>1148.895534</v>
       </c>
       <c r="G218" s="9">
-        <v>586.39299500000004</v>
+        <v>1148.895534</v>
       </c>
       <c r="H218" s="9">
         <v>1941.8589999999999</v>
@@ -19637,7 +19638,7 @@
         <v>1040.2974139999999</v>
       </c>
       <c r="G219" s="9">
-        <v>820.22796000000005</v>
+        <v>1040.2974139999999</v>
       </c>
       <c r="H219" s="9">
         <v>1957.249</v>
@@ -19669,7 +19670,7 @@
         <v>306.53069699999998</v>
       </c>
       <c r="G220" s="9">
-        <v>768.60185899999999</v>
+        <v>306.53069699999998</v>
       </c>
       <c r="H220" s="9">
         <v>2368.7939999999999</v>
@@ -19701,7 +19702,7 @@
         <v>127.12958500000001</v>
       </c>
       <c r="G221" s="9">
-        <v>147.16841600000001</v>
+        <v>127.12958500000001</v>
       </c>
       <c r="H221" s="9">
         <v>2247.54</v>
@@ -19733,7 +19734,7 @@
         <v>50.326332000000001</v>
       </c>
       <c r="G222" s="9">
-        <v>107.98893200000001</v>
+        <v>50.326332000000001</v>
       </c>
       <c r="H222" s="9">
         <v>2252.5500000000002</v>
@@ -19765,7 +19766,7 @@
         <v>142.668667</v>
       </c>
       <c r="G223" s="9">
-        <v>36.309688999999999</v>
+        <v>142.668667</v>
       </c>
       <c r="H223" s="9">
         <v>2413.3110000000001</v>
@@ -19797,7 +19798,7 @@
         <v>374.873828</v>
       </c>
       <c r="G224" s="9">
-        <v>4.0000000000000003E-5</v>
+        <v>374.873828</v>
       </c>
       <c r="H224" s="9">
         <v>2964.1610000000001</v>
@@ -19829,7 +19830,7 @@
         <v>880.05204900000001</v>
       </c>
       <c r="G225" s="9">
-        <v>2.5000000000000001E-5</v>
+        <v>880.05204900000001</v>
       </c>
       <c r="H225" s="9">
         <v>4261.4049999999997</v>
@@ -19861,7 +19862,7 @@
         <v>1782.7472600000001</v>
       </c>
       <c r="G226" s="9">
-        <v>0</v>
+        <v>1782.7472600000001</v>
       </c>
       <c r="H226" s="9">
         <v>3046.779</v>
@@ -19893,7 +19894,7 @@
         <v>1952.3405230000001</v>
       </c>
       <c r="G227" s="9">
-        <v>0.16200000000000001</v>
+        <v>1952.3405230000001</v>
       </c>
       <c r="H227" s="9">
         <v>2995.5030000000002</v>
@@ -19925,7 +19926,7 @@
         <v>1767.096372</v>
       </c>
       <c r="G228" s="9">
-        <v>71.959040000000002</v>
+        <v>1767.096372</v>
       </c>
       <c r="H228" s="9">
         <v>2485.7829999999999</v>
@@ -19957,7 +19958,7 @@
         <v>1642.7720890000001</v>
       </c>
       <c r="G229" s="9">
-        <v>530.09497399999998</v>
+        <v>1642.7720890000001</v>
       </c>
       <c r="H229" s="9">
         <v>2462.145</v>
@@ -19989,7 +19990,7 @@
         <v>1321.3496829999999</v>
       </c>
       <c r="G230" s="9">
-        <v>561.51926900000001</v>
+        <v>1321.3496829999999</v>
       </c>
       <c r="H230" s="9">
         <v>2152.86</v>
@@ -20021,7 +20022,7 @@
         <v>1607.039869</v>
       </c>
       <c r="G231" s="9">
-        <v>533.41717100000005</v>
+        <v>1607.039869</v>
       </c>
       <c r="H231" s="9">
         <v>2032.932</v>
@@ -20053,7 +20054,7 @@
         <v>1648.6252930000001</v>
       </c>
       <c r="G232" s="9">
-        <v>607.68507099999999</v>
+        <v>1648.6252930000001</v>
       </c>
       <c r="H232" s="9">
         <v>2402.3130000000001</v>
@@ -20085,7 +20086,7 @@
         <v>1400.992491</v>
       </c>
       <c r="G233" s="9">
-        <v>280.53807899999998</v>
+        <v>1400.992491</v>
       </c>
       <c r="H233" s="9">
         <v>2906.2570000000001</v>
@@ -20117,7 +20118,7 @@
         <v>1109.531367</v>
       </c>
       <c r="G234" s="9">
-        <v>68.141380999999996</v>
+        <v>1109.531367</v>
       </c>
       <c r="H234" s="9">
         <v>2722.3130000000001</v>
@@ -20149,7 +20150,7 @@
         <v>1385.183589</v>
       </c>
       <c r="G235" s="9">
-        <v>0</v>
+        <v>1385.183589</v>
       </c>
       <c r="H235" s="9">
         <v>2358.2629999999999</v>
@@ -20181,7 +20182,7 @@
         <v>821.39738</v>
       </c>
       <c r="G236" s="9">
-        <v>4.6999999999999997E-5</v>
+        <v>821.39738</v>
       </c>
       <c r="H236" s="9">
         <v>3149.357</v>
@@ -20213,7 +20214,7 @@
         <v>1205.0361760000001</v>
       </c>
       <c r="G237" s="9">
-        <v>0.18901000000000001</v>
+        <v>1205.0361760000001</v>
       </c>
       <c r="H237" s="9">
         <v>2428.0140000000001</v>
@@ -20245,7 +20246,7 @@
         <v>1309.3453939999999</v>
       </c>
       <c r="G238" s="9">
-        <v>0</v>
+        <v>1309.3453939999999</v>
       </c>
       <c r="H238" s="9">
         <v>3334.7710000000002</v>
@@ -20277,7 +20278,7 @@
         <v>1294.790407</v>
       </c>
       <c r="G239" s="9">
-        <v>7.3500040000000002</v>
+        <v>1294.790407</v>
       </c>
       <c r="H239" s="9">
         <v>3118.6120000000001</v>
@@ -20309,7 +20310,7 @@
         <v>1278.2356</v>
       </c>
       <c r="G240" s="9">
-        <v>0</v>
+        <v>1278.2356</v>
       </c>
       <c r="H240" s="9">
         <v>2866.585</v>
@@ -20341,7 +20342,7 @@
         <v>1714.60241</v>
       </c>
       <c r="G241" s="9">
-        <v>295.32080500000001</v>
+        <v>1714.60241</v>
       </c>
       <c r="H241" s="9">
         <v>3329.364</v>
@@ -20373,7 +20374,7 @@
         <v>1601.852052</v>
       </c>
       <c r="G242" s="9">
-        <v>935.03128100000004</v>
+        <v>1601.852052</v>
       </c>
       <c r="H242" s="9">
         <v>3605.828</v>
@@ -20405,7 +20406,7 @@
         <v>2555.6482369999999</v>
       </c>
       <c r="G243" s="9">
-        <v>274.200715</v>
+        <v>2555.6482369999999</v>
       </c>
       <c r="H243" s="9">
         <v>3101.277</v>
@@ -20437,7 +20438,7 @@
         <v>2070.0596829999999</v>
       </c>
       <c r="G244" s="9">
-        <v>830.25437499999998</v>
+        <v>2070.0596829999999</v>
       </c>
       <c r="H244" s="9">
         <v>3210.5810000000001</v>
@@ -20469,7 +20470,7 @@
         <v>1936.038716</v>
       </c>
       <c r="G245" s="9">
-        <v>362.61908599999998</v>
+        <v>1936.038716</v>
       </c>
       <c r="H245" s="9">
         <v>2465.46</v>
@@ -20501,7 +20502,7 @@
         <v>1650.5360310000001</v>
       </c>
       <c r="G246" s="9">
-        <v>55.018763</v>
+        <v>1650.5360310000001</v>
       </c>
       <c r="H246" s="9">
         <v>2326.89</v>
@@ -20533,7 +20534,7 @@
         <v>977.10214900000005</v>
       </c>
       <c r="G247" s="9">
-        <v>25.873121999999999</v>
+        <v>977.10214900000005</v>
       </c>
       <c r="H247" s="9">
         <v>2635.6680000000001</v>
@@ -20565,7 +20566,7 @@
         <v>1546.021675</v>
       </c>
       <c r="G248" s="9">
-        <v>5.0884799999999997</v>
+        <v>1546.021675</v>
       </c>
       <c r="H248" s="9">
         <v>2997.8440000000001</v>
@@ -20597,7 +20598,7 @@
         <v>2237.2078390000001</v>
       </c>
       <c r="G249" s="9">
-        <v>0</v>
+        <v>2237.2078390000001</v>
       </c>
       <c r="H249" s="9">
         <v>2627.0990000000002</v>
@@ -20629,7 +20630,7 @@
         <v>2315.393552</v>
       </c>
       <c r="G250" s="9">
-        <v>8.0000000000000007E-5</v>
+        <v>2315.393552</v>
       </c>
       <c r="H250" s="9">
         <v>2102.2919999999999</v>
@@ -20661,7 +20662,7 @@
         <v>1643.6218309999999</v>
       </c>
       <c r="G251" s="9">
-        <v>2.6999999999999999E-5</v>
+        <v>1643.6218309999999</v>
       </c>
       <c r="H251" s="9">
         <v>2121.7649999999999</v>
@@ -20693,7 +20694,7 @@
         <v>1329.6287090000001</v>
       </c>
       <c r="G252" s="9">
-        <v>1.0003E-2</v>
+        <v>1329.6287090000001</v>
       </c>
       <c r="H252" s="9">
         <v>2115.9369999999999</v>
@@ -20725,7 +20726,7 @@
         <v>800.61409400000002</v>
       </c>
       <c r="G253" s="9">
-        <v>344.244596</v>
+        <v>800.61409400000002</v>
       </c>
       <c r="H253" s="9">
         <v>1594.027</v>
@@ -20757,7 +20758,7 @@
         <v>888.65970500000003</v>
       </c>
       <c r="G254" s="9">
-        <v>551.67898700000001</v>
+        <v>888.65970500000003</v>
       </c>
       <c r="H254" s="9">
         <v>1641.425</v>
@@ -20789,7 +20790,7 @@
         <v>1179.183401</v>
       </c>
       <c r="G255" s="9">
-        <v>628.32881299999997</v>
+        <v>1179.183401</v>
       </c>
       <c r="H255" s="9">
         <v>2005.8530000000001</v>
@@ -20821,7 +20822,7 @@
         <v>1129.722714</v>
       </c>
       <c r="G256" s="9">
-        <v>246.89762500000001</v>
+        <v>1129.722714</v>
       </c>
       <c r="H256" s="9">
         <v>2191.6089999999999</v>
@@ -20853,7 +20854,7 @@
         <v>771.38830099999996</v>
       </c>
       <c r="G257" s="9">
-        <v>101.309766</v>
+        <v>771.38830099999996</v>
       </c>
       <c r="H257" s="9">
         <v>2217.2089999999998</v>
@@ -20885,7 +20886,7 @@
         <v>959.76996899999995</v>
       </c>
       <c r="G258" s="9">
-        <v>8.7999999999999998E-5</v>
+        <v>959.76996899999995</v>
       </c>
       <c r="H258" s="9">
         <v>2037.2750000000001</v>
@@ -20917,7 +20918,7 @@
         <v>825.47139900000002</v>
       </c>
       <c r="G259" s="9">
-        <v>0</v>
+        <v>825.47139900000002</v>
       </c>
       <c r="H259" s="9">
         <v>1643.9359999999999</v>
@@ -20949,7 +20950,7 @@
         <v>732.81323299999997</v>
       </c>
       <c r="G260" s="9">
-        <v>3.6999999999999998E-5</v>
+        <v>732.81323299999997</v>
       </c>
       <c r="H260" s="9">
         <v>2272.395</v>
@@ -20981,7 +20982,7 @@
         <v>1890.9359959999999</v>
       </c>
       <c r="G261" s="9">
-        <v>4.0000000000000003E-5</v>
+        <v>1890.9359959999999</v>
       </c>
       <c r="H261" s="9">
         <v>3002.7930000000001</v>
@@ -21013,7 +21014,7 @@
         <v>2094.383613</v>
       </c>
       <c r="G262" s="9">
-        <v>1.5999999999999999E-5</v>
+        <v>2094.383613</v>
       </c>
       <c r="H262" s="9">
         <v>3149.1619999999998</v>
@@ -21045,7 +21046,7 @@
         <v>1480.3831849999999</v>
       </c>
       <c r="G263" s="9">
-        <v>0</v>
+        <v>1480.3831849999999</v>
       </c>
       <c r="H263" s="9">
         <v>2529.8020000000001</v>
@@ -21077,7 +21078,7 @@
         <v>1076.258325</v>
       </c>
       <c r="G264" s="9">
-        <v>116.160656</v>
+        <v>1076.258325</v>
       </c>
       <c r="H264" s="9">
         <v>2230.4270000000001</v>
@@ -21109,7 +21110,7 @@
         <v>586.34568999999999</v>
       </c>
       <c r="G265" s="9">
-        <v>639.703575</v>
+        <v>586.34568999999999</v>
       </c>
       <c r="H265" s="9">
         <v>2246.692</v>
@@ -21141,7 +21142,7 @@
         <v>536.20427199999995</v>
       </c>
       <c r="G266" s="9">
-        <v>370.58351599999997</v>
+        <v>536.20427199999995</v>
       </c>
       <c r="H266" s="9">
         <v>2184.0790000000002</v>
@@ -21173,13 +21174,15 @@
         <v>637.91715299999998</v>
       </c>
       <c r="G267" s="9">
-        <v>226.706064</v>
+        <v>637.91715299999998</v>
       </c>
       <c r="H267" s="52"/>
       <c r="I267" s="9">
-        <v>2092.7420000000002</v>
-      </c>
-      <c r="J267" s="20"/>
+        <v>2060.92</v>
+      </c>
+      <c r="J267" s="52">
+        <v>6.6999279999999999</v>
+      </c>
     </row>
     <row r="268" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A268" s="20" t="s">
@@ -21194,15 +21197,19 @@
       <c r="D268" s="9">
         <v>1821.2739999999999</v>
       </c>
-      <c r="E268" s="20"/>
+      <c r="E268" s="71">
+        <v>2022.846</v>
+      </c>
       <c r="F268" s="9">
         <v>868.57358699999997</v>
       </c>
       <c r="G268" s="9">
-        <v>447.38076100000001</v>
+        <v>868.57358699999997</v>
       </c>
       <c r="H268" s="52"/>
-      <c r="I268" s="9"/>
+      <c r="I268" s="9">
+        <v>2159.5630000000001</v>
+      </c>
       <c r="J268" s="20"/>
     </row>
     <row r="269" spans="1:10" x14ac:dyDescent="0.25">
@@ -21222,7 +21229,9 @@
       <c r="F269" s="19">
         <v>892</v>
       </c>
-      <c r="G269" s="19"/>
+      <c r="G269" s="71">
+        <v>1297.6996959999999</v>
+      </c>
       <c r="H269" s="63"/>
       <c r="I269" s="19"/>
       <c r="J269" s="62"/>
@@ -21278,7 +21287,7 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -21286,7 +21295,7 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -21294,7 +21303,7 @@
         <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -21302,7 +21311,7 @@
         <v>6</v>
       </c>
       <c r="B5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -21579,26 +21588,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1f7db2c8-69c4-412b-9d44-16b2d9ce1096">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="2ae6f4a5-fc03-40a6-a6be-1c00f8eb7500" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100400F3C6901D84A48B91A9B4E5E69DA02" ma:contentTypeVersion="33" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="6ce5aaaf5c71f332bad539ea18ca4307">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1f7db2c8-69c4-412b-9d44-16b2d9ce1096" xmlns:ns3="2ae6f4a5-fc03-40a6-a6be-1c00f8eb7500" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="17518e73f766de7285d2370906e601ed" ns2:_="" ns3:_="">
     <xsd:import namespace="1f7db2c8-69c4-412b-9d44-16b2d9ce1096"/>
@@ -21859,10 +21848,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1f7db2c8-69c4-412b-9d44-16b2d9ce1096">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="2ae6f4a5-fc03-40a6-a6be-1c00f8eb7500" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{18313436-0D0C-4509-B8F8-BF1D4EE350A4}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DDC9D9EA-6611-4E83-9F93-4C0BB8E7E62A}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="1f7db2c8-69c4-412b-9d44-16b2d9ce1096"/>
+    <ds:schemaRef ds:uri="2ae6f4a5-fc03-40a6-a6be-1c00f8eb7500"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -21879,20 +21899,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DDC9D9EA-6611-4E83-9F93-4C0BB8E7E62A}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{18313436-0D0C-4509-B8F8-BF1D4EE350A4}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="1f7db2c8-69c4-412b-9d44-16b2d9ce1096"/>
-    <ds:schemaRef ds:uri="2ae6f4a5-fc03-40a6-a6be-1c00f8eb7500"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>